<commit_message>
I fix the augmentation amount.
</commit_message>
<xml_diff>
--- a/labeled/Add_Eating/July/classification_results.xlsx
+++ b/labeled/Add_Eating/July/classification_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D431"/>
+  <dimension ref="A1:D430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -689,7 +689,7 @@
         <v>0</v>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
         <v>0</v>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -788,7 +788,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
         <v>0</v>
       </c>
       <c r="B34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -2183,7 +2183,7 @@
         <v>0</v>
       </c>
       <c r="B98" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
         <v>0</v>
       </c>
       <c r="B114" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2705,7 @@
         <v>0</v>
       </c>
       <c r="B127" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -2738,19 +2738,19 @@
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
         <v>1</v>
       </c>
       <c r="B131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C131" t="inlineStr">
         <is>
@@ -2786,7 +2786,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
         <v>1</v>
       </c>
       <c r="B144" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C144" t="inlineStr">
         <is>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
         <v>1</v>
       </c>
       <c r="B155" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C155" t="inlineStr">
         <is>
@@ -3218,7 +3218,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
         <v>1</v>
       </c>
       <c r="B159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C159" t="inlineStr">
         <is>
@@ -3290,7 +3290,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3515,7 @@
         <v>1</v>
       </c>
       <c r="B172" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C172" t="inlineStr">
         <is>
@@ -3524,7 +3524,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3695,7 @@
         <v>1</v>
       </c>
       <c r="B182" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C182" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -4487,7 +4487,7 @@
         <v>1</v>
       </c>
       <c r="B226" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C226" t="inlineStr">
         <is>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -4595,7 +4595,7 @@
         <v>1</v>
       </c>
       <c r="B232" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C232" t="inlineStr">
         <is>
@@ -4604,7 +4604,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -4721,7 +4721,7 @@
         <v>1</v>
       </c>
       <c r="B239" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C239" t="inlineStr">
         <is>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4757,7 @@
         <v>1</v>
       </c>
       <c r="B241" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C241" t="inlineStr">
         <is>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -4829,7 +4829,7 @@
         <v>1</v>
       </c>
       <c r="B245" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C245" t="inlineStr">
         <is>
@@ -4838,7 +4838,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -4865,7 +4865,7 @@
         <v>1</v>
       </c>
       <c r="B247" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C247" t="inlineStr">
         <is>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -4973,7 +4973,7 @@
         <v>1</v>
       </c>
       <c r="B253" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C253" t="inlineStr">
         <is>
@@ -4982,7 +4982,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
         <v>1</v>
       </c>
       <c r="B259" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C259" t="inlineStr">
         <is>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -5117,7 +5117,7 @@
         <v>1</v>
       </c>
       <c r="B261" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C261" t="inlineStr">
         <is>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -5171,7 +5171,7 @@
         <v>1</v>
       </c>
       <c r="B264" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C264" t="inlineStr">
         <is>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -5297,7 +5297,7 @@
         <v>1</v>
       </c>
       <c r="B271" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C271" t="inlineStr">
         <is>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -5438,14 +5438,14 @@
     </row>
     <row r="279">
       <c r="A279" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B279" t="n">
         <v>1</v>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -5693,7 +5693,7 @@
         <v>2</v>
       </c>
       <c r="B293" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C293" t="inlineStr">
         <is>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5801,7 @@
         <v>2</v>
       </c>
       <c r="B299" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C299" t="inlineStr">
         <is>
@@ -5810,7 +5810,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -5909,7 +5909,7 @@
         <v>2</v>
       </c>
       <c r="B305" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C305" t="inlineStr">
         <is>
@@ -5918,7 +5918,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -6035,7 +6035,7 @@
         <v>2</v>
       </c>
       <c r="B312" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C312" t="inlineStr">
         <is>
@@ -6044,7 +6044,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -6053,7 +6053,7 @@
         <v>2</v>
       </c>
       <c r="B313" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C313" t="inlineStr">
         <is>
@@ -6062,7 +6062,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -6071,7 +6071,7 @@
         <v>2</v>
       </c>
       <c r="B314" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C314" t="inlineStr">
         <is>
@@ -6080,7 +6080,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -6107,7 +6107,7 @@
         <v>2</v>
       </c>
       <c r="B316" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C316" t="inlineStr">
         <is>
@@ -6116,7 +6116,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -6143,7 +6143,7 @@
         <v>2</v>
       </c>
       <c r="B318" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C318" t="inlineStr">
         <is>
@@ -6152,7 +6152,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -6197,7 +6197,7 @@
         <v>2</v>
       </c>
       <c r="B321" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C321" t="inlineStr">
         <is>
@@ -6206,7 +6206,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -6233,7 +6233,7 @@
         <v>2</v>
       </c>
       <c r="B323" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C323" t="inlineStr">
         <is>
@@ -6242,7 +6242,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -6251,7 +6251,7 @@
         <v>2</v>
       </c>
       <c r="B324" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C324" t="inlineStr">
         <is>
@@ -6260,7 +6260,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -6341,7 +6341,7 @@
         <v>2</v>
       </c>
       <c r="B329" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C329" t="inlineStr">
         <is>
@@ -6350,7 +6350,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -6377,7 +6377,7 @@
         <v>2</v>
       </c>
       <c r="B331" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C331" t="inlineStr">
         <is>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -6395,7 +6395,7 @@
         <v>2</v>
       </c>
       <c r="B332" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C332" t="inlineStr">
         <is>
@@ -6404,7 +6404,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -6431,7 +6431,7 @@
         <v>2</v>
       </c>
       <c r="B334" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C334" t="inlineStr">
         <is>
@@ -6440,7 +6440,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -6503,7 +6503,7 @@
         <v>2</v>
       </c>
       <c r="B338" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C338" t="inlineStr">
         <is>
@@ -6512,7 +6512,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -6719,7 +6719,7 @@
         <v>2</v>
       </c>
       <c r="B350" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C350" t="inlineStr">
         <is>
@@ -6728,7 +6728,7 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -6881,7 +6881,7 @@
         <v>2</v>
       </c>
       <c r="B359" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C359" t="inlineStr">
         <is>
@@ -6890,7 +6890,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -6935,7 +6935,7 @@
         <v>2</v>
       </c>
       <c r="B362" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C362" t="inlineStr">
         <is>
@@ -6944,7 +6944,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -7007,7 +7007,7 @@
         <v>2</v>
       </c>
       <c r="B366" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C366" t="inlineStr">
         <is>
@@ -7016,7 +7016,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -7043,7 +7043,7 @@
         <v>2</v>
       </c>
       <c r="B368" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C368" t="inlineStr">
         <is>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -7187,7 +7187,7 @@
         <v>2</v>
       </c>
       <c r="B376" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C376" t="inlineStr">
         <is>
@@ -7196,7 +7196,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -7367,7 +7367,7 @@
         <v>2</v>
       </c>
       <c r="B386" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C386" t="inlineStr">
         <is>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -7529,7 +7529,7 @@
         <v>2</v>
       </c>
       <c r="B395" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C395" t="inlineStr">
         <is>
@@ -7538,7 +7538,7 @@
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7565,7 @@
         <v>2</v>
       </c>
       <c r="B397" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C397" t="inlineStr">
         <is>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -7601,7 +7601,7 @@
         <v>2</v>
       </c>
       <c r="B399" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C399" t="inlineStr">
         <is>
@@ -7610,7 +7610,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -7655,7 +7655,7 @@
         <v>2</v>
       </c>
       <c r="B402" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C402" t="inlineStr">
         <is>
@@ -7664,7 +7664,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -7709,7 +7709,7 @@
         <v>2</v>
       </c>
       <c r="B405" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C405" t="inlineStr">
         <is>
@@ -7718,7 +7718,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -7781,7 +7781,7 @@
         <v>2</v>
       </c>
       <c r="B409" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C409" t="inlineStr">
         <is>
@@ -7790,7 +7790,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -7799,7 +7799,7 @@
         <v>2</v>
       </c>
       <c r="B410" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C410" t="inlineStr">
         <is>
@@ -7808,7 +7808,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -7835,7 +7835,7 @@
         <v>2</v>
       </c>
       <c r="B412" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C412" t="inlineStr">
         <is>
@@ -7844,7 +7844,7 @@
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -7853,7 +7853,7 @@
         <v>2</v>
       </c>
       <c r="B413" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C413" t="inlineStr">
         <is>
@@ -7862,7 +7862,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -7925,7 +7925,7 @@
         <v>2</v>
       </c>
       <c r="B417" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C417" t="inlineStr">
         <is>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -8051,7 +8051,7 @@
         <v>2</v>
       </c>
       <c r="B424" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C424" t="inlineStr">
         <is>
@@ -8060,7 +8060,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -8167,24 +8167,6 @@
         </is>
       </c>
       <c r="D430" t="inlineStr">
-        <is>
-          <t>Eating</t>
-        </is>
-      </c>
-    </row>
-    <row r="431">
-      <c r="A431" t="n">
-        <v>2</v>
-      </c>
-      <c r="B431" t="n">
-        <v>2</v>
-      </c>
-      <c r="C431" t="inlineStr">
-        <is>
-          <t>Eating</t>
-        </is>
-      </c>
-      <c r="D431" t="inlineStr">
         <is>
           <t>Eating</t>
         </is>

</xml_diff>

<commit_message>
after a long time
</commit_message>
<xml_diff>
--- a/labeled/Add_Eating/July/classification_results.xlsx
+++ b/labeled/Add_Eating/July/classification_results.xlsx
@@ -689,7 +689,7 @@
         <v>0</v>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
         <v>0</v>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -788,7 +788,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
         <v>0</v>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1193,7 @@
         <v>0</v>
       </c>
       <c r="B43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2417,7 @@
         <v>0</v>
       </c>
       <c r="B111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2705,7 @@
         <v>0</v>
       </c>
       <c r="B127" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -2993,7 +2993,7 @@
         <v>1</v>
       </c>
       <c r="B143" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C143" t="inlineStr">
         <is>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3011,7 @@
         <v>1</v>
       </c>
       <c r="B144" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C144" t="inlineStr">
         <is>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
         <v>1</v>
       </c>
       <c r="B154" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C154" t="inlineStr">
         <is>
@@ -3200,7 +3200,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
         <v>1</v>
       </c>
       <c r="B155" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C155" t="inlineStr">
         <is>
@@ -3218,7 +3218,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3695,7 @@
         <v>1</v>
       </c>
       <c r="B182" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C182" t="inlineStr">
         <is>
@@ -3704,7 +3704,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -4253,7 +4253,7 @@
         <v>1</v>
       </c>
       <c r="B213" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C213" t="inlineStr">
         <is>
@@ -4262,7 +4262,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -4271,7 +4271,7 @@
         <v>1</v>
       </c>
       <c r="B214" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C214" t="inlineStr">
         <is>
@@ -4280,7 +4280,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -4487,7 +4487,7 @@
         <v>1</v>
       </c>
       <c r="B226" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C226" t="inlineStr">
         <is>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -5243,7 +5243,7 @@
         <v>1</v>
       </c>
       <c r="B268" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C268" t="inlineStr">
         <is>
@@ -5252,7 +5252,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -5477,7 +5477,7 @@
         <v>2</v>
       </c>
       <c r="B281" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C281" t="inlineStr">
         <is>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -5657,7 +5657,7 @@
         <v>2</v>
       </c>
       <c r="B291" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C291" t="inlineStr">
         <is>
@@ -5666,7 +5666,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -5675,7 +5675,7 @@
         <v>2</v>
       </c>
       <c r="B292" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C292" t="inlineStr">
         <is>
@@ -5684,7 +5684,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5801,7 @@
         <v>2</v>
       </c>
       <c r="B299" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C299" t="inlineStr">
         <is>
@@ -5810,7 +5810,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -6017,7 +6017,7 @@
         <v>2</v>
       </c>
       <c r="B311" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C311" t="inlineStr">
         <is>
@@ -6026,7 +6026,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -6125,7 +6125,7 @@
         <v>2</v>
       </c>
       <c r="B317" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C317" t="inlineStr">
         <is>
@@ -6134,7 +6134,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -6251,7 +6251,7 @@
         <v>2</v>
       </c>
       <c r="B324" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C324" t="inlineStr">
         <is>
@@ -6260,7 +6260,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -6269,7 +6269,7 @@
         <v>2</v>
       </c>
       <c r="B325" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C325" t="inlineStr">
         <is>
@@ -6278,7 +6278,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -6449,7 +6449,7 @@
         <v>2</v>
       </c>
       <c r="B335" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C335" t="inlineStr">
         <is>
@@ -6458,7 +6458,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -6593,7 +6593,7 @@
         <v>2</v>
       </c>
       <c r="B343" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C343" t="inlineStr">
         <is>
@@ -6602,7 +6602,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -6719,7 +6719,7 @@
         <v>2</v>
       </c>
       <c r="B350" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C350" t="inlineStr">
         <is>
@@ -6728,7 +6728,7 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -6737,7 +6737,7 @@
         <v>2</v>
       </c>
       <c r="B351" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C351" t="inlineStr">
         <is>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -6827,7 +6827,7 @@
         <v>2</v>
       </c>
       <c r="B356" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C356" t="inlineStr">
         <is>
@@ -6836,7 +6836,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -7781,7 +7781,7 @@
         <v>2</v>
       </c>
       <c r="B409" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C409" t="inlineStr">
         <is>
@@ -7790,7 +7790,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -7853,7 +7853,7 @@
         <v>2</v>
       </c>
       <c r="B413" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C413" t="inlineStr">
         <is>
@@ -7862,7 +7862,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>Not_Drinking</t>
+          <t>Eating</t>
         </is>
       </c>
     </row>
@@ -8033,7 +8033,7 @@
         <v>2</v>
       </c>
       <c r="B423" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C423" t="inlineStr">
         <is>
@@ -8042,7 +8042,7 @@
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>
@@ -8087,7 +8087,7 @@
         <v>2</v>
       </c>
       <c r="B426" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C426" t="inlineStr">
         <is>
@@ -8096,7 +8096,7 @@
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Drinking</t>
         </is>
       </c>
     </row>
@@ -8105,7 +8105,7 @@
         <v>2</v>
       </c>
       <c r="B427" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C427" t="inlineStr">
         <is>
@@ -8114,7 +8114,7 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Eating</t>
+          <t>Not_Drinking</t>
         </is>
       </c>
     </row>

</xml_diff>